<commit_message>
fix bug delete category
</commit_message>
<xml_diff>
--- a/public/PositionData/position2.xlsx
+++ b/public/PositionData/position2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>ID</t>
   </si>
@@ -27,13 +27,7 @@
     <t>Nama Posisi</t>
   </si>
   <si>
-    <t>Test Posisi baru 2</t>
-  </si>
-  <si>
-    <t>Test Posisi baru 3</t>
-  </si>
-  <si>
-    <t>Test Posisi baru 4</t>
+    <t>Test Posisi baru 1000</t>
   </si>
 </sst>
 </file>
@@ -406,21 +400,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
       <c r="L4" s="1"/>
     </row>
   </sheetData>

</xml_diff>